<commit_message>
Fix: correctly flag redundant items as Tier 4 in installation_priority.xlsx
</commit_message>
<xml_diff>
--- a/AI_SYSTEMS_INVENTORY/installation_priority.xlsx
+++ b/AI_SYSTEMS_INVENTORY/installation_priority.xlsx
@@ -1166,7 +1166,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>seo-audit</t>
+          <t>copywriting</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>copywriting</t>
+          <t>email-sequence</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1242,28 +1242,28 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>email-sequence</t>
+          <t>canvas-design / image-enhancer / slack-gif-creator / video-downloader</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Skill (Community)</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>claude-skills</t>
+          <t>awesome-claude-skills</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
         <v>3.2</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1280,28 +1280,28 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>canvas-design / image-enhancer / slack-gif-creator / video-downloader</t>
+          <t>content-batch + /content-batch command</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Skill (Community)</t>
+          <t>Skill+Command</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>awesome-claude-skills</t>
+          <t>claude-marketing</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
         <v>3.2</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>4</v>
+        <v>6.5</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1318,24 +1318,24 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>content-batch + /content-batch command</t>
+          <t>social-content</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Skill+Command</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>claude-marketing</t>
+          <t>claude-skills</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>6.5</v>
+        <v>6.2</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
@@ -1356,17 +1356,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>social-content</t>
+          <t>page-cro / signup-flow-cro / form-cro / popup-cro / paywall-upgrade-cro / onboarding-cro</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Skill Bundle</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>claude-skills</t>
+          <t>claude-marketing</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>page-cro / signup-flow-cro / form-cro / popup-cro / paywall-upgrade-cro / onboarding-cro</t>
+          <t>Web/Mobile/Dashboard Prototype skills</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Skill Bundle</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>claude-marketing</t>
+          <t>open-design</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
@@ -1432,12 +1432,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Web/Mobile/Dashboard Prototype skills</t>
+          <t>Automations (scheduled design generation)</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Feature</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1470,24 +1470,24 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Automations (scheduled design generation)</t>
+          <t>graphify (AST + LLM knowledge graph)</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>CLI/Skill</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>open-design</t>
+          <t>graphify</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>6.2</v>
+        <v>6</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
@@ -1508,17 +1508,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>graphify (AST + LLM knowledge graph)</t>
+          <t>stripe-automation / shopify-automation</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>CLI/Skill</t>
+          <t>Skill (Composio)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>graphify</t>
+          <t>awesome-claude-skills</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
@@ -1546,24 +1546,24 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>stripe-automation / shopify-automation</t>
+          <t>docx / pdf / pptx / xlsx (anthropics canonical)</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Skill (Composio)</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>awesome-claude-skills</t>
+          <t>skills</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
@@ -1584,17 +1584,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>docx / pdf / pptx / xlsx (official Anthropic)</t>
+          <t>Bring-Your-Own-Agent (22+ coding agents) + MCP server</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>awesome-claude-skills</t>
+          <t>open-design</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
@@ -1622,24 +1622,24 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>docx / pdf / pptx / xlsx (anthropics canonical)</t>
+          <t>figma-automation / canva (Composio)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Skill</t>
+          <t>Skill (Composio)</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>skills</t>
+          <t>awesome-claude-skills</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
@@ -1660,24 +1660,24 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Bring-Your-Own-Agent (22+ coding agents) + MCP server</t>
+          <t>content-research-writer / lead-research-assistant / twitter-algorithm-optimizer</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Skill (Community)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>open-design</t>
+          <t>awesome-claude-skills</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
@@ -1698,17 +1698,17 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>figma-automation / canva (Composio)</t>
+          <t>Data Formulator app (Data/Chart Agents)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Skill (Composio)</t>
+          <t>Application</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>awesome-claude-skills</t>
+          <t>data-formulator</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -1736,24 +1736,24 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>content-research-writer / lead-research-assistant / twitter-algorithm-optimizer</t>
+          <t>mem-search / search MCP tool</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Skill (Community)</t>
+          <t>MCP Tool</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>awesome-claude-skills</t>
+          <t>claude-mem</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
@@ -1774,24 +1774,24 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Data Formulator app (Data/Chart Agents)</t>
+          <t>graphify query / explain / path</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Application</t>
+          <t>CLI</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>data-formulator</t>
+          <t>graphify</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
@@ -1812,24 +1812,24 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>mem-search / search MCP tool</t>
+          <t>MCP stdio/HTTP servers</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>MCP Tool</t>
+          <t>MCP Server</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>claude-mem</t>
+          <t>graphify</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
@@ -1850,24 +1850,24 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>graphify query / explain / path</t>
+          <t>churn-prevention + analytics-tracking + ab-test-setup</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>CLI</t>
+          <t>Skill Bundle</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>graphify</t>
+          <t>claude-marketing</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
@@ -1888,17 +1888,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>MCP stdio/HTTP servers</t>
+          <t>Deck templates (15 designs / 36 themes)</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>MCP Server</t>
+          <t>Skill</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>graphify</t>
+          <t>open-design</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
@@ -1919,78 +1919,78 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Tier 3 - Optional</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>churn-prevention + analytics-tracking + ab-test-setup</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Skill Bundle</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>claude-marketing</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F39" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Tier 4 - Skip</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>seo-audit</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>claude-skills</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>Useful for specific workflows but niche, high-complexity, or low-frequency - install on demand.</t>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Redundant - duplicate/overlap with a higher-rated tool (see redundancy_analysis.xlsx). Skip to avoid maintenance overhead.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Tier 3 - Optional</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Deck templates (15 designs / 36 themes)</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Tier 4 - Skip</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>docx / pdf / pptx / xlsx (official Anthropic)</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Skill</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>open-design</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F40" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>awesome-claude-skills</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>Useful for specific workflows but niche, high-complexity, or low-frequency - install on demand.</t>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Redundant - duplicate/overlap with a higher-rated tool (see redundancy_analysis.xlsx). Skip to avoid maintenance overhead.</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="H59" s="5" t="inlineStr">
         <is>
-          <t>Low priority score - high complexity relative to value, or covered by another tool. Safe to skip initially.</t>
+          <t>Redundant - duplicate/overlap with a higher-rated tool (see redundancy_analysis.xlsx). Skip to avoid maintenance overhead.</t>
         </is>
       </c>
     </row>

</xml_diff>